<commit_message>
Update screening merge with revised 조선·기자재 and assignee names
- 조선·기자재: HD현대마린솔루션 탈락 사유를 업종 평균 PER·PBR 대비
  배수 비교로 다시 쓴 수정본 반영
- 담당자 기재: 방산·우주 심규환 / 2차전지·소재·소프트웨어 배준서
- 팀 1은 담당 산업 6개에 인원 4명(배준서 2개 겸임, 지주는 팀 2 팀장)
  이라는 점을 취합 시트에 표기

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jphTyMQLHbxpFNoQ68jkL
</commit_message>
<xml_diff>
--- a/docs/26-2/data/ICOK_1팀_담당산업_스크리닝.xlsx
+++ b/docs/26-2/data/ICOK_1팀_담당산업_스크리닝.xlsx
@@ -1187,9 +1187,9 @@
           <t>2차전지·소재</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>미기재</t>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>배준서</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1216,9 +1216,9 @@
           <t>소프트웨어·인터넷·게임</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>미기재</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>배준서</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>배준서</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>배준서</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1691,7 +1691,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>2차전지·소재 · 소프트웨어·인터넷·게임 · 지주는 담당자와 제출일이 비어 있다. 팀장이 확인한다.</t>
+          <t>배준서 팀장이 2차전지·소재와 소프트웨어·인터넷·게임 2개를 겸임한다. 지주는 팀 2 팀장이 맡았으므로 담당 산업 6개에 팀 1 인원은 4명이다. 1인 1산업 전제가 성립하지 않는다.</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,11 @@
           <t>담당자</t>
         </is>
       </c>
-      <c r="E4" s="34" t="n"/>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>배준서</t>
+        </is>
+      </c>
       <c r="F4" s="35" t="n"/>
       <c r="G4" s="30" t="inlineStr">
         <is>
@@ -7758,7 +7762,11 @@
           <t>담당자</t>
         </is>
       </c>
-      <c r="E4" s="34" t="n"/>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>배준서</t>
+        </is>
+      </c>
       <c r="F4" s="35" t="n"/>
       <c r="G4" s="30" t="inlineStr">
         <is>

</xml_diff>